<commit_message>
chore: Update TranslationMapping.xlsx with new translations
</commit_message>
<xml_diff>
--- a/TranslationMapping.xlsx
+++ b/TranslationMapping.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roma0050\Documents\projects\digidiggie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B9F477-5F67-42F6-8242-E46AC5683F9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{45CF3B26-1CB2-4A60-9ED4-00869AC0AB41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="255" yWindow="285" windowWidth="28545" windowHeight="16995" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1890" yWindow="113" windowWidth="24022" windowHeight="15922" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TranslationMapping" sheetId="3" r:id="rId1"/>
     <sheet name="TableMapping" sheetId="6" r:id="rId2"/>
-    <sheet name="Queries" sheetId="7" r:id="rId3"/>
-    <sheet name="RowSource" sheetId="8" r:id="rId4"/>
-    <sheet name="RowSourceCompute" sheetId="2" r:id="rId5"/>
-    <sheet name="Gudrun" sheetId="5" r:id="rId6"/>
+    <sheet name="Expressions" sheetId="9" r:id="rId3"/>
+    <sheet name="Queries" sheetId="7" r:id="rId4"/>
+    <sheet name="RowSource" sheetId="8" r:id="rId5"/>
+    <sheet name="RowSourceCompute" sheetId="2" r:id="rId6"/>
+    <sheet name="Gudrun" sheetId="5" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="communities">TranslationMapping!$A$2:$F$4</definedName>
     <definedName name="entries">TranslationMapping!$A$5:$F$20</definedName>
-    <definedName name="Externadata_1" localSheetId="5" hidden="1">Gudrun!$A$1:$G$54</definedName>
+    <definedName name="Externadata_1" localSheetId="6" hidden="1">Gudrun!$A$1:$G$54</definedName>
     <definedName name="judgements">TranslationMapping!$A$53:$F$54</definedName>
     <definedName name="land_use">TranslationMapping!$A$24:$F$25</definedName>
     <definedName name="legal_sources">TranslationMapping!$A$45:$F$46</definedName>
@@ -37,6 +38,7 @@
     <definedName name="winners">TranslationMapping!$A$49:$F$50</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -206,7 +208,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="259">
   <si>
     <t>ID</t>
   </si>
@@ -971,6 +973,18 @@
   </si>
   <si>
     <t>[Ortnamn_ny]</t>
+  </si>
+  <si>
+    <t>[given_name] &amp; " " &amp; [PATRONYME] &amp; " " &amp; [Tillnamn] &amp; " " &amp; [Född] &amp; "-" &amp; [Död] &amp; " " &amp; [Bynamn]</t>
+  </si>
+  <si>
+    <t>OriginalExpression</t>
+  </si>
+  <si>
+    <t>[given_name] &amp; " " &amp; [patronymic] &amp; " " &amp; [surname] &amp; " " &amp; [birth_year] &amp; "-" &amp; [death_year] &amp; " " &amp; [community_name]</t>
+  </si>
+  <si>
+    <t>TranslatedExpression</t>
   </si>
 </sst>
 </file>
@@ -1191,9 +1205,9 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1583,7 +1597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EFBBA10-227A-4C3E-97E2-4D28C36FEBA2}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="15.86328125" style="12" bestFit="1" customWidth="1"/>
@@ -1592,10 +1606,11 @@
     <col min="4" max="4" width="17.265625" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="104.59765625" style="5" customWidth="1"/>
     <col min="6" max="6" width="14.1328125" style="18" customWidth="1"/>
-    <col min="7" max="16384" width="9.1328125" style="5"/>
+    <col min="7" max="7" width="34.86328125" style="5" customWidth="1"/>
+    <col min="8" max="16384" width="9.1328125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>166</v>
       </c>
@@ -1614,8 +1629,11 @@
       <c r="F1" s="15" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G1" s="29" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>245</v>
       </c>
@@ -1633,7 +1651,7 @@
       </c>
       <c r="F2" s="16"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="6" t="s">
         <v>245</v>
       </c>
@@ -1651,7 +1669,7 @@
       </c>
       <c r="F3" s="16"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="6" t="s">
         <v>245</v>
       </c>
@@ -1669,7 +1687,7 @@
       </c>
       <c r="F4" s="16"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
         <v>246</v>
       </c>
@@ -1687,7 +1705,7 @@
       </c>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="13" t="s">
         <v>246</v>
       </c>
@@ -1705,7 +1723,7 @@
       </c>
       <c r="F6" s="16"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="6" t="s">
         <v>246</v>
       </c>
@@ -1723,7 +1741,7 @@
       </c>
       <c r="F7" s="16"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="6" t="s">
         <v>246</v>
       </c>
@@ -1741,7 +1759,7 @@
       </c>
       <c r="F8" s="16"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="6" t="s">
         <v>246</v>
       </c>
@@ -1759,7 +1777,7 @@
       </c>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
         <v>246</v>
       </c>
@@ -1777,7 +1795,7 @@
       </c>
       <c r="F10" s="16"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
         <v>246</v>
       </c>
@@ -1795,7 +1813,7 @@
       </c>
       <c r="F11" s="16"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="6" t="s">
         <v>246</v>
       </c>
@@ -1813,7 +1831,7 @@
       </c>
       <c r="F12" s="16"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
         <v>246</v>
       </c>
@@ -1831,7 +1849,7 @@
       </c>
       <c r="F13" s="16"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="6" t="s">
         <v>246</v>
       </c>
@@ -1849,7 +1867,7 @@
       </c>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
         <v>246</v>
       </c>
@@ -1867,7 +1885,7 @@
       </c>
       <c r="F15" s="16"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>246</v>
       </c>
@@ -2179,7 +2197,7 @@
       </c>
       <c r="F32" s="16"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A33" s="6" t="s">
         <v>249</v>
       </c>
@@ -2199,7 +2217,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A34" s="6" t="s">
         <v>249</v>
       </c>
@@ -2217,7 +2235,7 @@
       </c>
       <c r="F34" s="16"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A35" s="6" t="s">
         <v>249</v>
       </c>
@@ -2237,7 +2255,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A36" s="6" t="s">
         <v>249</v>
       </c>
@@ -2257,7 +2275,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A37" s="6" t="s">
         <v>249</v>
       </c>
@@ -2277,7 +2295,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A38" s="6" t="s">
         <v>249</v>
       </c>
@@ -2295,7 +2313,7 @@
       </c>
       <c r="F38" s="16"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A39" s="6" t="s">
         <v>249</v>
       </c>
@@ -2315,7 +2333,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" s="6" t="s">
         <v>249</v>
       </c>
@@ -2335,7 +2353,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A41" s="6" t="s">
         <v>249</v>
       </c>
@@ -2355,7 +2373,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A42" s="6" t="s">
         <v>249</v>
       </c>
@@ -2373,7 +2391,7 @@
       </c>
       <c r="F42" s="16"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A43" s="6" t="s">
         <v>249</v>
       </c>
@@ -2393,7 +2411,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A44" s="6" t="s">
         <v>249</v>
       </c>
@@ -2410,8 +2428,11 @@
         <v>133</v>
       </c>
       <c r="F44" s="16"/>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G44" s="5" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A45" s="6" t="s">
         <v>250</v>
       </c>
@@ -2429,7 +2450,7 @@
       </c>
       <c r="F45" s="16"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A46" s="6" t="s">
         <v>250</v>
       </c>
@@ -2447,7 +2468,7 @@
       </c>
       <c r="F46" s="16"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A47" s="6" t="s">
         <v>206</v>
       </c>
@@ -2465,7 +2486,7 @@
       </c>
       <c r="F47" s="16"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A48" s="6" t="s">
         <v>206</v>
       </c>
@@ -2878,6 +2899,65 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B510BD7-0F12-4758-A514-20641236A78C}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.06640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="82.265625" customWidth="1"/>
+    <col min="6" max="6" width="99" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="F1" s="25" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{367B9837-7527-4194-AAEA-9453D79A2611}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2886,7 +2966,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C881608D-D1C8-4511-9254-FFF1593EF725}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -3107,7 +3187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93093E98-6D8B-4028-8401-3861BC40C700}">
   <dimension ref="A1:K41"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
@@ -3177,7 +3257,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B3" s="5" t="s">
@@ -3203,7 +3283,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -3229,7 +3309,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -3255,7 +3335,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -3281,7 +3361,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B7" s="5" t="s">
@@ -3307,7 +3387,7 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B8" s="5" t="s">
@@ -3333,7 +3413,7 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A9" s="27" t="s">
+      <c r="A9" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B9" s="5" t="s">
@@ -3359,7 +3439,7 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A10" s="27" t="s">
+      <c r="A10" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -3385,7 +3465,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A11" s="27" t="s">
+      <c r="A11" s="5" t="s">
         <v>246</v>
       </c>
       <c r="B11" s="5" t="s">
@@ -3954,261 +4034,261 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A30" s="29" t="s">
+      <c r="A30" s="28" t="s">
         <v>166</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C30" s="28" t="s">
         <v>182</v>
       </c>
-      <c r="D30" s="29" t="s">
+      <c r="D30" s="28" t="s">
         <v>183</v>
       </c>
-      <c r="E30" s="29" t="s">
+      <c r="E30" s="28" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A31" s="28" t="str">
-        <f>A2</f>
+      <c r="A31" s="27" t="str">
+        <f t="shared" ref="A31:B41" si="11">A2</f>
         <v>[Byar]</v>
       </c>
-      <c r="B31" s="28" t="str">
-        <f>B2</f>
+      <c r="B31" s="27" t="str">
+        <f t="shared" si="11"/>
         <v>[Socken]</v>
       </c>
-      <c r="C31" s="28" t="str">
-        <f>A17</f>
+      <c r="C31" s="27" t="str">
+        <f t="shared" ref="C31:C41" si="12">A17</f>
         <v>communities</v>
       </c>
-      <c r="D31" s="28" t="str">
-        <f ca="1">B17</f>
+      <c r="D31" s="27" t="str">
+        <f t="shared" ref="D31:D41" ca="1" si="13">B17</f>
         <v>parish_id</v>
       </c>
-      <c r="E31" s="28" t="str">
+      <c r="E31" s="27" t="str">
         <f ca="1">I17</f>
         <v>SELECT [parishes].[parish_id], [parishes].[parish] FROM [parishes] ORDER BY [parish]</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A32" s="28" t="str">
-        <f t="shared" ref="A32:B32" si="11">A3</f>
+      <c r="A32" s="27" t="str">
+        <f t="shared" si="11"/>
         <v>[Entries]</v>
       </c>
-      <c r="B32" s="28" t="str">
+      <c r="B32" s="27" t="str">
         <f t="shared" si="11"/>
         <v>[Aktör]</v>
       </c>
-      <c r="C32" s="28" t="str">
-        <f t="shared" ref="C32:D32" si="12">A18</f>
+      <c r="C32" s="27" t="str">
+        <f t="shared" si="12"/>
         <v>entries</v>
       </c>
-      <c r="D32" s="28" t="str">
-        <f t="shared" ca="1" si="12"/>
+      <c r="D32" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
         <v>actor_id</v>
       </c>
-      <c r="E32" s="28" t="str">
-        <f t="shared" ref="E32:E41" ca="1" si="13">I18</f>
+      <c r="E32" s="27" t="str">
+        <f t="shared" ref="E32:E41" ca="1" si="14">I18</f>
         <v>SELECT [persons].[person_id], [persons].[full_name] FROM [persons] ORDER BY [full_name]</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A33" s="28" t="str">
-        <f t="shared" ref="A33:B33" si="14">A4</f>
+      <c r="A33" s="27" t="str">
+        <f t="shared" si="11"/>
         <v>[Entries]</v>
       </c>
-      <c r="B33" s="28" t="str">
+      <c r="B33" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[By]</v>
+      </c>
+      <c r="C33" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D33" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>community_id</v>
+      </c>
+      <c r="E33" s="27" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v>SELECT [communities].[community_id], [communities].[community_name] FROM [communities] ORDER BY [community_name]</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Entries]</v>
+      </c>
+      <c r="B34" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Källa]</v>
+      </c>
+      <c r="C34" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D34" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>source_id</v>
+      </c>
+      <c r="E34" s="27" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v>SELECT [sources].[source_id], [sources].[source_abbreviation] FROM [sources] ORDER BY [source_abbreviation]</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Entries]</v>
+      </c>
+      <c r="B35" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Årstid2]</v>
+      </c>
+      <c r="C35" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D35" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>season_id</v>
+      </c>
+      <c r="E35" s="27" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v>SELECT [seasons].[season_id], [seasons].[season_name] FROM [seasons] ORDER BY [season_name]</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Entries]</v>
+      </c>
+      <c r="B36" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Resurs]</v>
+      </c>
+      <c r="C36" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D36" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>land_use_id</v>
+      </c>
+      <c r="E36" s="27" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v>SELECT [land_use].[land_use_id], [land_use].[type] FROM [land_use] ORDER BY [type]</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Entries]</v>
+      </c>
+      <c r="B37" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Vinnare]</v>
+      </c>
+      <c r="C37" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D37" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>winner_id</v>
+      </c>
+      <c r="E37" s="27" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v>SELECT [winners].[winner_id], [winners].[winner_description] FROM [winners] ORDER BY [winner_description]</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Entries]</v>
+      </c>
+      <c r="B38" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Rättskälla]</v>
+      </c>
+      <c r="C38" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D38" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>legal_source_id</v>
+      </c>
+      <c r="E38" s="27" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v>SELECT [legal_sources].[legal_source_id], [legal_sources].[legal_source_name] FROM [legal_sources] ORDER BY [legal_source_name]</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Entries]</v>
+      </c>
+      <c r="B39" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Dom]</v>
+      </c>
+      <c r="C39" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D39" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>judgement_id</v>
+      </c>
+      <c r="E39" s="27" t="str">
+        <f t="shared" ca="1" si="14"/>
+        <v>SELECT [judgements].[judgement_id], [judgements].[sanction] FROM [judgements] ORDER BY [sanction]</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Entries]</v>
+      </c>
+      <c r="B40" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Ortnamn]</v>
+      </c>
+      <c r="C40" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>entries</v>
+      </c>
+      <c r="D40" s="27" t="str">
+        <f t="shared" ca="1" si="13"/>
+        <v>placename_id</v>
+      </c>
+      <c r="E40" s="27" t="str">
         <f t="shared" si="14"/>
-        <v>[By]</v>
-      </c>
-      <c r="C33" s="28" t="str">
-        <f t="shared" ref="C33:D33" si="15">A19</f>
-        <v>entries</v>
-      </c>
-      <c r="D33" s="28" t="str">
-        <f t="shared" ca="1" si="15"/>
-        <v>community_id</v>
-      </c>
-      <c r="E33" s="28" t="str">
+        <v>SELECT [Ortnamn_ny1].[ID], [Ortnamn_ny1].[Kombo] FROM Ortnamn_ny1 ORDER BY [Kombo];</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A41" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Personer]</v>
+      </c>
+      <c r="B41" s="27" t="str">
+        <f t="shared" si="11"/>
+        <v>[Bynamn]</v>
+      </c>
+      <c r="C41" s="27" t="str">
+        <f t="shared" si="12"/>
+        <v>persons</v>
+      </c>
+      <c r="D41" s="27" t="str">
         <f t="shared" ca="1" si="13"/>
-        <v>SELECT [communities].[community_id], [communities].[community_name] FROM [communities] ORDER BY [community_name]</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A34" s="28" t="str">
-        <f t="shared" ref="A34:B34" si="16">A5</f>
-        <v>[Entries]</v>
-      </c>
-      <c r="B34" s="28" t="str">
-        <f t="shared" si="16"/>
-        <v>[Källa]</v>
-      </c>
-      <c r="C34" s="28" t="str">
-        <f t="shared" ref="C34:D34" si="17">A20</f>
-        <v>entries</v>
-      </c>
-      <c r="D34" s="28" t="str">
-        <f t="shared" ca="1" si="17"/>
-        <v>source_id</v>
-      </c>
-      <c r="E34" s="28" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v>SELECT [sources].[source_id], [sources].[source_abbreviation] FROM [sources] ORDER BY [source_abbreviation]</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A35" s="28" t="str">
-        <f t="shared" ref="A35:B35" si="18">A6</f>
-        <v>[Entries]</v>
-      </c>
-      <c r="B35" s="28" t="str">
-        <f t="shared" si="18"/>
-        <v>[Årstid2]</v>
-      </c>
-      <c r="C35" s="28" t="str">
-        <f t="shared" ref="C35:D35" si="19">A21</f>
-        <v>entries</v>
-      </c>
-      <c r="D35" s="28" t="str">
-        <f t="shared" ca="1" si="19"/>
-        <v>season_id</v>
-      </c>
-      <c r="E35" s="28" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v>SELECT [seasons].[season_id], [seasons].[season_name] FROM [seasons] ORDER BY [season_name]</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A36" s="28" t="str">
-        <f t="shared" ref="A36:B36" si="20">A7</f>
-        <v>[Entries]</v>
-      </c>
-      <c r="B36" s="28" t="str">
-        <f t="shared" si="20"/>
-        <v>[Resurs]</v>
-      </c>
-      <c r="C36" s="28" t="str">
-        <f t="shared" ref="C36:D36" si="21">A22</f>
-        <v>entries</v>
-      </c>
-      <c r="D36" s="28" t="str">
-        <f t="shared" ca="1" si="21"/>
-        <v>land_use_id</v>
-      </c>
-      <c r="E36" s="28" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v>SELECT [land_use].[land_use_id], [land_use].[type] FROM [land_use] ORDER BY [type]</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A37" s="28" t="str">
-        <f t="shared" ref="A37:B37" si="22">A8</f>
-        <v>[Entries]</v>
-      </c>
-      <c r="B37" s="28" t="str">
-        <f t="shared" si="22"/>
-        <v>[Vinnare]</v>
-      </c>
-      <c r="C37" s="28" t="str">
-        <f t="shared" ref="C37:D37" si="23">A23</f>
-        <v>entries</v>
-      </c>
-      <c r="D37" s="28" t="str">
-        <f t="shared" ca="1" si="23"/>
-        <v>winner_id</v>
-      </c>
-      <c r="E37" s="28" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v>SELECT [winners].[winner_id], [winners].[winner_description] FROM [winners] ORDER BY [winner_description]</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A38" s="28" t="str">
-        <f t="shared" ref="A38:B38" si="24">A9</f>
-        <v>[Entries]</v>
-      </c>
-      <c r="B38" s="28" t="str">
-        <f t="shared" si="24"/>
-        <v>[Rättskälla]</v>
-      </c>
-      <c r="C38" s="28" t="str">
-        <f t="shared" ref="C38:D38" si="25">A24</f>
-        <v>entries</v>
-      </c>
-      <c r="D38" s="28" t="str">
-        <f t="shared" ca="1" si="25"/>
-        <v>legal_source_id</v>
-      </c>
-      <c r="E38" s="28" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v>SELECT [legal_sources].[legal_source_id], [legal_sources].[legal_source_name] FROM [legal_sources] ORDER BY [legal_source_name]</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A39" s="28" t="str">
-        <f t="shared" ref="A39:B39" si="26">A10</f>
-        <v>[Entries]</v>
-      </c>
-      <c r="B39" s="28" t="str">
-        <f t="shared" si="26"/>
-        <v>[Dom]</v>
-      </c>
-      <c r="C39" s="28" t="str">
-        <f t="shared" ref="C39:D39" si="27">A25</f>
-        <v>entries</v>
-      </c>
-      <c r="D39" s="28" t="str">
-        <f t="shared" ca="1" si="27"/>
-        <v>judgement_id</v>
-      </c>
-      <c r="E39" s="28" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v>SELECT [judgements].[judgement_id], [judgements].[sanction] FROM [judgements] ORDER BY [sanction]</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A40" s="28" t="str">
-        <f t="shared" ref="A40:B40" si="28">A11</f>
-        <v>[Entries]</v>
-      </c>
-      <c r="B40" s="28" t="str">
-        <f t="shared" si="28"/>
-        <v>[Ortnamn]</v>
-      </c>
-      <c r="C40" s="28" t="str">
-        <f t="shared" ref="C40:D40" si="29">A26</f>
-        <v>entries</v>
-      </c>
-      <c r="D40" s="28" t="str">
-        <f t="shared" ca="1" si="29"/>
-        <v>placename_id</v>
-      </c>
-      <c r="E40" s="28" t="str">
-        <f t="shared" si="13"/>
-        <v>SELECT [Ortnamn_ny1].[ID], [Ortnamn_ny1].[Kombo] FROM Ortnamn_ny1 ORDER BY [Kombo];</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A41" s="28" t="str">
-        <f t="shared" ref="A41:B41" si="30">A12</f>
-        <v>[Personer]</v>
-      </c>
-      <c r="B41" s="28" t="str">
-        <f t="shared" si="30"/>
-        <v>[Bynamn]</v>
-      </c>
-      <c r="C41" s="28" t="str">
-        <f t="shared" ref="C41:D41" si="31">A27</f>
-        <v>persons</v>
-      </c>
-      <c r="D41" s="28" t="str">
-        <f t="shared" ca="1" si="31"/>
         <v>community_name</v>
       </c>
-      <c r="E41" s="28" t="str">
-        <f t="shared" si="13"/>
+      <c r="E41" s="27" t="str">
+        <f t="shared" si="14"/>
         <v>SELECT [communities].[community_name] FROM [communities] ORDER BY [community_name];</v>
       </c>
     </row>
@@ -4219,7 +4299,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7980C792-44BF-4C5C-A9E8-C9CD7AE83411}">
   <dimension ref="A1:H54"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
chore: Update TranslationMapping.xlsx with new data
</commit_message>
<xml_diff>
--- a/TranslationMapping.xlsx
+++ b/TranslationMapping.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roma0050\Documents\projects\digidiggie\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45CF3B26-1CB2-4A60-9ED4-00869AC0AB41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EBBCB2-A867-49A5-8332-9E4396975F4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1890" yWindow="113" windowWidth="24022" windowHeight="15922" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1890" yWindow="113" windowWidth="24022" windowHeight="15922" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TranslationMapping" sheetId="3" r:id="rId1"/>
-    <sheet name="TableMapping" sheetId="6" r:id="rId2"/>
-    <sheet name="Expressions" sheetId="9" r:id="rId3"/>
-    <sheet name="Queries" sheetId="7" r:id="rId4"/>
-    <sheet name="RowSource" sheetId="8" r:id="rId5"/>
+    <sheet name="QueryDefinitions" sheetId="7" r:id="rId2"/>
+    <sheet name="RowSource" sheetId="8" r:id="rId3"/>
+    <sheet name="TableMapping" sheetId="6" r:id="rId4"/>
+    <sheet name="Expressions" sheetId="9" r:id="rId5"/>
     <sheet name="RowSourceCompute" sheetId="2" r:id="rId6"/>
     <sheet name="Gudrun" sheetId="5" r:id="rId7"/>
   </sheets>
@@ -38,7 +38,6 @@
     <definedName name="winners">TranslationMapping!$A$49:$F$50</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -208,7 +207,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="263">
   <si>
     <t>ID</t>
   </si>
@@ -981,10 +980,44 @@
     <t>OriginalExpression</t>
   </si>
   <si>
-    <t>[given_name] &amp; " " &amp; [patronymic] &amp; " " &amp; [surname] &amp; " " &amp; [birth_year] &amp; "-" &amp; [death_year] &amp; " " &amp; [community_name]</t>
-  </si>
-  <si>
     <t>TranslatedExpression</t>
+  </si>
+  <si>
+    <t>QueryName</t>
+  </si>
+  <si>
+    <t>SQLText</t>
+  </si>
+  <si>
+    <t>SELECT
+    [persons].[full_name],
+    [communities].[community_name],
+    [entries].[year],
+    [entries].[description],
+    [land_use].[type],
+    [seasons].[season_name],
+    [entries].[land_rights_status],
+    [entries].[original_placename],
+    [community_names].[Ortnamn],
+    [sources].[source_abbreviation],
+    [entries].[reference_number],
+    [community_names].[LOPNR],
+    [community_names].[N],
+    [community_names].[E],
+    [entries].[ID]
+FROM ( ( ( ( ( sources
+INNER JOIN entries ON [sources].[source_id] = [entries].[source_id] )
+INNER JOIN seasons ON [seasons].[season_id] = [entries].[season_id] )
+INNER JOIN land_use ON [land_use].[land_use_id] = [entries].[resource_id] )
+INNER JOIN communities ON [communities].[community_id] = [entries].[community_id] )
+INNER JOIN persons ON [persons].[person_id] = [entries].[actor_id] )
+INNER JOIN community_names ON community_names.[ID] = entries.[placename_id];</t>
+  </si>
+  <si>
+    <t>event_query</t>
+  </si>
+  <si>
+    <t>[given_name] &amp; ' ' &amp; [patronymic] &amp; ' ' &amp; [surname] &amp; ' ' &amp; [birth_year] &amp; '-' &amp; [death_year] &amp; ' ' &amp; [community_name]</t>
   </si>
 </sst>
 </file>
@@ -1167,7 +1200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1208,6 +1241,12 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1606,7 +1645,7 @@
     <col min="4" max="4" width="17.265625" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="104.59765625" style="5" customWidth="1"/>
     <col min="6" max="6" width="14.1328125" style="18" customWidth="1"/>
-    <col min="7" max="7" width="34.86328125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="94.46484375" style="5" customWidth="1"/>
     <col min="8" max="16384" width="9.1328125" style="5"/>
   </cols>
   <sheetData>
@@ -1630,7 +1669,7 @@
         <v>179</v>
       </c>
       <c r="G1" s="29" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.4">
@@ -2411,7 +2450,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
         <v>249</v>
       </c>
@@ -2428,8 +2467,8 @@
         <v>133</v>
       </c>
       <c r="F44" s="16"/>
-      <c r="G44" s="5" t="s">
-        <v>257</v>
+      <c r="G44" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.4">
@@ -2620,6 +2659,256 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{367B9837-7527-4194-AAEA-9453D79A2611}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="73.3984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="330.4" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="30" t="s">
+        <v>261</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>260</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C881608D-D1C8-4511-9254-FFF1593EF725}">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.06640625" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="106.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A1" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="25" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B4" t="s">
+        <v>208</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B5" t="s">
+        <v>212</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>246</v>
+      </c>
+      <c r="B6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" t="s">
+        <v>217</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B9" t="s">
+        <v>218</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>246</v>
+      </c>
+      <c r="B10" t="s">
+        <v>219</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>246</v>
+      </c>
+      <c r="B11" t="s">
+        <v>220</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" t="s">
+        <v>205</v>
+      </c>
+      <c r="C12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" t="s">
+        <v>161</v>
+      </c>
+      <c r="E12" t="s">
+        <v>201</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED6CEF77-4FE4-4B8F-9014-B148E5EFEFE5}">
   <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2898,7 +3187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B510BD7-0F12-4758-A514-20641236A78C}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2928,7 +3217,7 @@
         <v>256</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
@@ -2948,242 +3237,12 @@
         <v>255</v>
       </c>
       <c r="F2" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{367B9837-7527-4194-AAEA-9453D79A2611}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C881608D-D1C8-4511-9254-FFF1593EF725}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="11.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.06640625" customWidth="1"/>
-    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="106.06640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A1" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="B1" s="25" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="25" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="25" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>245</v>
-      </c>
-      <c r="B2" t="s">
-        <v>206</v>
-      </c>
-      <c r="C2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>246</v>
-      </c>
-      <c r="B3" t="s">
-        <v>207</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>246</v>
-      </c>
-      <c r="B4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>160</v>
-      </c>
-      <c r="E4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>246</v>
-      </c>
-      <c r="B5" t="s">
-        <v>212</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>246</v>
-      </c>
-      <c r="B6" t="s">
-        <v>214</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>246</v>
-      </c>
-      <c r="B7" t="s">
-        <v>215</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E7" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>246</v>
-      </c>
-      <c r="B8" t="s">
-        <v>217</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" t="s">
-        <v>49</v>
-      </c>
-      <c r="E8" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>246</v>
-      </c>
-      <c r="B9" t="s">
-        <v>218</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
-        <v>52</v>
-      </c>
-      <c r="E9" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>246</v>
-      </c>
-      <c r="B10" t="s">
-        <v>219</v>
-      </c>
-      <c r="C10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>246</v>
-      </c>
-      <c r="B11" t="s">
-        <v>220</v>
-      </c>
-      <c r="C11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>249</v>
-      </c>
-      <c r="B12" t="s">
-        <v>205</v>
-      </c>
-      <c r="C12" t="s">
-        <v>79</v>
-      </c>
-      <c r="D12" t="s">
-        <v>161</v>
-      </c>
-      <c r="E12" t="s">
-        <v>201</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>